<commit_message>
fixed for haneen error
</commit_message>
<xml_diff>
--- a/static/marchMadness/2026/ExcelBrackets/haneen-march-madness-bracket-2026.xlsx
+++ b/static/marchMadness/2026/ExcelBrackets/haneen-march-madness-bracket-2026.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_9D2382D991E35D0B505D16462B27D42DF56B2394" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE0EE556-4F9B-4200-AA78-750017D0FF4B}"/>
+  <bookViews>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="madness" state="visible" r:id="rId4"/>
+    <sheet name="madness" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="78">
   <si>
     <t>2026 March Madness Bracket</t>
   </si>
@@ -134,9 +138,6 @@
   </si>
   <si>
     <t>Queens</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Michigan</t>
@@ -253,14 +254,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -623,16 +624,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AM72"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:38" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -667,7 +668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B7">
         <v>1</v>
       </c>
@@ -681,7 +682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E8" t="s">
         <v>7</v>
       </c>
@@ -689,7 +690,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B9">
         <v>16</v>
       </c>
@@ -703,7 +704,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H10" t="s">
         <v>7</v>
       </c>
@@ -711,7 +712,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B11">
         <v>8</v>
       </c>
@@ -725,7 +726,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E12" t="s">
         <v>13</v>
       </c>
@@ -733,7 +734,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B13">
         <v>9</v>
       </c>
@@ -747,7 +748,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K14" t="s">
         <v>7</v>
       </c>
@@ -755,7 +756,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B15">
         <v>5</v>
       </c>
@@ -769,7 +770,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E16" t="s">
         <v>15</v>
       </c>
@@ -777,7 +778,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B17">
         <v>12</v>
       </c>
@@ -791,7 +792,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H18" t="s">
         <v>19</v>
       </c>
@@ -799,7 +800,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B19">
         <v>4</v>
       </c>
@@ -813,7 +814,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E20" t="s">
         <v>19</v>
       </c>
@@ -821,7 +822,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B21">
         <v>13</v>
       </c>
@@ -835,7 +836,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K22" t="s">
         <v>23</v>
       </c>
@@ -849,7 +850,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B23">
         <v>6</v>
       </c>
@@ -863,7 +864,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E24" t="s">
         <v>27</v>
       </c>
@@ -871,7 +872,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B25">
         <v>11</v>
       </c>
@@ -885,7 +886,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H26" t="s">
         <v>29</v>
       </c>
@@ -893,7 +894,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B27">
         <v>3</v>
       </c>
@@ -907,7 +908,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E28" t="s">
         <v>29</v>
       </c>
@@ -915,7 +916,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B29">
         <v>14</v>
       </c>
@@ -929,7 +930,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K30" t="s">
         <v>33</v>
       </c>
@@ -937,7 +938,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B31">
         <v>7</v>
       </c>
@@ -951,7 +952,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E32" t="s">
         <v>34</v>
       </c>
@@ -959,7 +960,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B33">
         <v>10</v>
       </c>
@@ -973,7 +974,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H34" t="s">
         <v>33</v>
       </c>
@@ -981,7 +982,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B35">
         <v>2</v>
       </c>
@@ -995,7 +996,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E36" t="s">
         <v>33</v>
       </c>
@@ -1003,7 +1004,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B37">
         <v>15</v>
       </c>
@@ -1017,371 +1018,371 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="15:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="O39" t="s">
+        <v>7</v>
+      </c>
+      <c r="W39" t="s">
         <v>41</v>
       </c>
-      <c r="W39" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="42" spans="2:39" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AL42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="AM42">
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AJ43" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="2:39" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B44">
         <v>16</v>
       </c>
       <c r="C44" t="s">
+        <v>43</v>
+      </c>
+      <c r="R44" t="s">
+        <v>41</v>
+      </c>
+      <c r="AL44" t="s">
         <v>44</v>
-      </c>
-      <c r="R44" t="s">
-        <v>42</v>
-      </c>
-      <c r="AL44" t="s">
-        <v>45</v>
       </c>
       <c r="AM44">
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AG45" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="46" spans="2:39" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B46">
         <v>8</v>
       </c>
       <c r="C46" t="s">
+        <v>45</v>
+      </c>
+      <c r="R46" t="s">
         <v>46</v>
       </c>
-      <c r="R46" t="s">
+      <c r="AL46" t="s">
         <v>47</v>
-      </c>
-      <c r="AL46" t="s">
-        <v>48</v>
       </c>
       <c r="AM46">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="AJ47" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="48" spans="2:39" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="48" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B48">
         <v>9</v>
       </c>
       <c r="C48" t="s">
+        <v>48</v>
+      </c>
+      <c r="AL48" t="s">
         <v>49</v>
-      </c>
-      <c r="AL48" t="s">
-        <v>50</v>
       </c>
       <c r="AM48">
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K49" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AD49" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="50" spans="2:39" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="50" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B50">
         <v>5</v>
       </c>
       <c r="C50" t="s">
+        <v>50</v>
+      </c>
+      <c r="S50" t="s">
         <v>51</v>
       </c>
-      <c r="S50" t="s">
+      <c r="AL50" t="s">
         <v>52</v>
-      </c>
-      <c r="AL50" t="s">
-        <v>53</v>
       </c>
       <c r="AM50">
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AJ51" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="52" spans="2:39" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="52" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B52">
         <v>12</v>
       </c>
       <c r="C52" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AL52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AM52">
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H53" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AG53" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="54" spans="2:39" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="54" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B54">
         <v>4</v>
       </c>
       <c r="C54" t="s">
+        <v>56</v>
+      </c>
+      <c r="R54" t="s">
         <v>57</v>
       </c>
-      <c r="R54" t="s">
-        <v>58</v>
-      </c>
       <c r="AL54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AM54">
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E55" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AJ55" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="56" spans="2:39" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="56" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B56">
         <v>13</v>
       </c>
       <c r="C56" t="s">
+        <v>58</v>
+      </c>
+      <c r="AL56" t="s">
         <v>59</v>
-      </c>
-      <c r="AL56" t="s">
-        <v>60</v>
       </c>
       <c r="AM56">
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K57" t="s">
+        <v>60</v>
+      </c>
+      <c r="N57" t="s">
         <v>61</v>
       </c>
-      <c r="N57" t="s">
+      <c r="AA57" t="s">
+        <v>41</v>
+      </c>
+      <c r="AD57" t="s">
         <v>62</v>
       </c>
-      <c r="AA57" t="s">
-        <v>42</v>
-      </c>
-      <c r="AD57" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="58" spans="2:39" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B58">
         <v>6</v>
       </c>
       <c r="C58" t="s">
+        <v>63</v>
+      </c>
+      <c r="AL58" t="s">
         <v>64</v>
-      </c>
-      <c r="AL58" t="s">
-        <v>65</v>
       </c>
       <c r="AM58">
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E59" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AJ59" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="60" spans="2:39" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="60" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B60">
         <v>11</v>
       </c>
       <c r="C60" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL60" t="s">
         <v>66</v>
-      </c>
-      <c r="AL60" t="s">
-        <v>67</v>
       </c>
       <c r="AM60">
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H61" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG61" t="s">
         <v>68</v>
       </c>
-      <c r="AG61" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="62" spans="2:39" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B62">
         <v>3</v>
       </c>
       <c r="C62" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL62" t="s">
         <v>68</v>
-      </c>
-      <c r="AL62" t="s">
-        <v>69</v>
       </c>
       <c r="AM62">
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E63" t="s">
+        <v>67</v>
+      </c>
+      <c r="AJ63" t="s">
         <v>68</v>
       </c>
-      <c r="AJ63" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="64" spans="2:39" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B64">
         <v>14</v>
       </c>
       <c r="C64" t="s">
+        <v>69</v>
+      </c>
+      <c r="AL64" t="s">
         <v>70</v>
-      </c>
-      <c r="AL64" t="s">
-        <v>71</v>
       </c>
       <c r="AM64">
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="11:30" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="K65" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AD65" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="66" spans="2:39" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="66" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B66">
         <v>7</v>
       </c>
       <c r="C66" t="s">
+        <v>72</v>
+      </c>
+      <c r="AL66" t="s">
         <v>73</v>
-      </c>
-      <c r="AL66" t="s">
-        <v>74</v>
       </c>
       <c r="AM66">
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E67" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AJ67" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="68" spans="2:39" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="68" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B68">
         <v>10</v>
       </c>
       <c r="C68" t="s">
+        <v>74</v>
+      </c>
+      <c r="AL68" t="s">
         <v>75</v>
-      </c>
-      <c r="AL68" t="s">
-        <v>76</v>
       </c>
       <c r="AM68">
         <v>10</v>
       </c>
     </row>
-    <row r="69" spans="8:33" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="H69" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG69" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="70" spans="2:39" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="70" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B70">
         <v>2</v>
       </c>
       <c r="C70" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AL70" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AM70">
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="5:36" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="E71" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AJ71" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="72" spans="2:39" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="72" spans="2:39" x14ac:dyDescent="0.55000000000000004">
       <c r="B72">
         <v>15</v>
       </c>
       <c r="C72" t="s">
+        <v>76</v>
+      </c>
+      <c r="AL72" t="s">
         <v>77</v>
-      </c>
-      <c r="AL72" t="s">
-        <v>78</v>
       </c>
       <c r="AM72">
         <v>15</v>
@@ -1389,6 +1390,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>